<commit_message>
data(objccc): objetivos Tradicional por vendedor actualizados (suman 845)
El usuario repartio los 36 objetivos Tradicional que faltaban asignar.
Ahora la hoja tradicional suma 845 exacto (antes 809) y coincide con el
Total declarado. objetivo_asignado == objetivo_total == 1046, asi que la
leyenda "sin asignar" del pie de la tarjeta se oculta sola.

Solo cambia el input objccc.xlsx; sin tocar server ni portal. Validado
en navegador + endpoint.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/01_INPUTS/objccc.xlsx
+++ b/01_INPUTS/objccc.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Orbit\MATINAL_PENAFLOR\01_INPUTS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0C3F0281-1627-42B0-AA4E-33BE46B36109}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F6FA06D1-6BCD-4EE6-AF0D-A8486C527187}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{472D008F-7292-4943-B105-A39854C23553}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" activeTab="3" xr2:uid="{472D008F-7292-4943-B105-A39854C23553}"/>
   </bookViews>
   <sheets>
     <sheet name="total" sheetId="1" r:id="rId1"/>
@@ -872,7 +872,7 @@
         <v>8</v>
       </c>
       <c r="D4" s="14">
-        <v>105</v>
+        <v>116</v>
       </c>
     </row>
     <row r="5" spans="2:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -883,7 +883,7 @@
         <v>9</v>
       </c>
       <c r="D5" s="14">
-        <v>114</v>
+        <v>118</v>
       </c>
     </row>
     <row r="6" spans="2:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -916,7 +916,7 @@
         <v>12</v>
       </c>
       <c r="D8" s="14">
-        <v>102</v>
+        <v>116</v>
       </c>
     </row>
     <row r="9" spans="2:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -927,7 +927,7 @@
         <v>13</v>
       </c>
       <c r="D9" s="14">
-        <v>110</v>
+        <v>117</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
data: objetivos actualizados (11T, CCC) + dadatinto
Primera publicacion por la via nueva del allowlist. Sin esto el fix del .bat no
se nota hasta el proximo cierre: Render seguiria con el objetivo 11T del 06/07
y el objccc del 21/07.

Objetivo 11T total: 1864 -> 3734 (los 11 titulares). OJO en la matinal: el % de
avance del 11T se corta casi al medio. Es el numero correcto, no una caida de
venta.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/01_INPUTS/objccc.xlsx
+++ b/01_INPUTS/objccc.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Orbit\MATINAL_PENAFLOR\01_INPUTS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F6FA06D1-6BCD-4EE6-AF0D-A8486C527187}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CF920486-CB0C-4954-99E7-680A14CDA110}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" activeTab="3" xr2:uid="{472D008F-7292-4943-B105-A39854C23553}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" activeTab="1" xr2:uid="{472D008F-7292-4943-B105-A39854C23553}"/>
   </bookViews>
   <sheets>
     <sheet name="total" sheetId="1" r:id="rId1"/>

</xml_diff>